<commit_message>
Update publication and award data; add new grant reporting and department awards files
- Updated `table_D4b_citations_by_publication_year.csv` to include total citations.
- Revised `table_F1_faculty_research_awards.csv` to specify competitive designations for awards.
- Modified `table_F2_grad_committee_mentoring_activity.csv` to reflect changes in committee memberships.
- Adjusted `table_G1_student_engagement_partial.csv` to correct student engagement data for 2026.
- Added new files: `grant_reporting_window_difference.csv` and `grant_total_reconciliation.csv` for grant reporting analysis.
- Introduced `table_F0_department_awards_by_year.csv` to track departmental awards over the years.
</commit_message>
<xml_diff>
--- a/data/awards.xlsx
+++ b/data/awards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://colostate.sharepoint.com/sites/CASDARETeam-5yearReview/Shared Documents/Research and Creative Artistry - LAUREN/dare_research/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{94E3764B-164D-42FC-8899-2391B8E340B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9D7B082-8DEB-40D5-A457-8FFBA2FDD13D}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{94E3764B-164D-42FC-8899-2391B8E340B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B99B30C4-6942-446A-8E16-318A9CDD18C5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A000FD71-334D-49A3-8CB4-C1C0AD911838}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="91">
   <si>
     <t>Year</t>
   </si>
@@ -98,9 +98,6 @@
     <t>College</t>
   </si>
   <si>
-    <t>CSU Empowering Community Engagement Scholarship Award (x3)</t>
-  </si>
-  <si>
     <t>Colorado State University</t>
   </si>
   <si>
@@ -221,12 +218,6 @@
     <t>AAEA Distinguished Extension/Outreach Program Award</t>
   </si>
   <si>
-    <t>Bruce Gardner Award (x2)</t>
-  </si>
-  <si>
-    <t>CAS Outstanding Emerging Community Engagement Scholarship Award (x2)</t>
-  </si>
-  <si>
     <t>Agricultural Experiment Station / CAS</t>
   </si>
   <si>
@@ -269,18 +260,9 @@
     <t>Charles N. Shepardson Instructional Innovation Award</t>
   </si>
   <si>
-    <t>Charles N. Shepardson Graduate Student Teaching Award (x2)</t>
-  </si>
-  <si>
     <t>Charles N. Shepardson Faculty Teaching Award (&lt; 10 yrs at CSU)</t>
   </si>
   <si>
-    <t>Excellence in Collaborative Research Award w/ AgNext (x2)</t>
-  </si>
-  <si>
-    <t>Charles N. Shepardson Student Leadership Award (x2)</t>
-  </si>
-  <si>
     <t>CAS Lincoln Laureate Award</t>
   </si>
   <si>
@@ -291,6 +273,45 @@
   </si>
   <si>
     <t>Dept / Assoc / Univ / National</t>
+  </si>
+  <si>
+    <t>CSU Empowering Community Engagement Scholarship Award (1 of 3)</t>
+  </si>
+  <si>
+    <t>CSU Empowering Community Engagement Scholarship Award (2 of 3)</t>
+  </si>
+  <si>
+    <t>CSU Empowering Community Engagement Scholarship Award (3 of 3)</t>
+  </si>
+  <si>
+    <t>Bruce Gardner Award (1 of 2)</t>
+  </si>
+  <si>
+    <t>Bruce Gardner Award (2 of 2)</t>
+  </si>
+  <si>
+    <t>CAS Outstanding Emerging Community Engagement Scholarship Award (1 of 2)</t>
+  </si>
+  <si>
+    <t>CAS Outstanding Emerging Community Engagement Scholarship Award (2 of 2)</t>
+  </si>
+  <si>
+    <t>Charles N. Shepardson Graduate Student Teaching Award (1 of 2)</t>
+  </si>
+  <si>
+    <t>Charles N. Shepardson Graduate Student Teaching Award (2 of 2)</t>
+  </si>
+  <si>
+    <t>Excellence in Collaborative Research Award w/ AgNext (1 of 2)</t>
+  </si>
+  <si>
+    <t>Excellence in Collaborative Research Award w/ AgNext (2 of 2)</t>
+  </si>
+  <si>
+    <t>Charles N. Shepardson Student Leadership Award (1 of 2)</t>
+  </si>
+  <si>
+    <t>Charles N. Shepardson Student Leadership Award (2 of 2)</t>
   </si>
 </sst>
 </file>
@@ -341,16 +362,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -685,35 +705,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D7BD42A-1F77-4096-AAA4-87BF19C9D574}">
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" style="2" customWidth="1"/>
-    <col min="2" max="2" width="54.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="35" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14" style="2" customWidth="1"/>
-    <col min="5" max="6" width="12" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="62.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>83</v>
+      <c r="D1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -821,19 +840,19 @@
         <v>2020</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -841,19 +860,19 @@
         <v>2020</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -861,19 +880,19 @@
         <v>2020</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -881,27 +900,27 @@
         <v>2020</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>16</v>
@@ -910,7 +929,7 @@
         <v>5</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>18</v>
@@ -918,22 +937,22 @@
     </row>
     <row r="12" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -941,30 +960,30 @@
         <v>2021</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>11</v>
@@ -973,18 +992,18 @@
         <v>6</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>11</v>
@@ -993,7 +1012,7 @@
         <v>6</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1001,19 +1020,19 @@
         <v>2022</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1021,10 +1040,10 @@
         <v>2022</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>11</v>
@@ -1033,7 +1052,7 @@
         <v>6</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1041,16 +1060,16 @@
         <v>2022</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>7</v>
@@ -1061,10 +1080,10 @@
         <v>2022</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>11</v>
@@ -1073,7 +1092,7 @@
         <v>6</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1081,19 +1100,19 @@
         <v>2022</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1101,19 +1120,19 @@
         <v>2022</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1121,19 +1140,19 @@
         <v>2022</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1141,19 +1160,19 @@
         <v>2022</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1161,19 +1180,19 @@
         <v>2022</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1181,19 +1200,19 @@
         <v>2022</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1201,19 +1220,19 @@
         <v>2022</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>7</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1221,33 +1240,33 @@
         <v>2022</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>6</v>
@@ -1258,22 +1277,22 @@
     </row>
     <row r="29" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1281,19 +1300,19 @@
         <v>2023</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1301,13 +1320,13 @@
         <v>2023</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>6</v>
@@ -1321,19 +1340,19 @@
         <v>2023</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1341,16 +1360,16 @@
         <v>2023</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>18</v>
@@ -1361,10 +1380,10 @@
         <v>2023</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>11</v>
@@ -1381,13 +1400,13 @@
         <v>2023</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>12</v>
@@ -1401,16 +1420,16 @@
         <v>2023</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>7</v>
@@ -1418,33 +1437,33 @@
     </row>
     <row r="37" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>11</v>
@@ -1461,19 +1480,19 @@
         <v>2024</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>62</v>
+        <v>4</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1481,19 +1500,19 @@
         <v>2024</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>62</v>
+        <v>4</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1501,19 +1520,19 @@
         <v>2024</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>62</v>
+        <v>4</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1521,19 +1540,19 @@
         <v>2024</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1541,16 +1560,16 @@
         <v>2024</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>18</v>
@@ -1561,13 +1580,13 @@
         <v>2024</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>6</v>
@@ -1581,36 +1600,36 @@
         <v>2024</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>7</v>
@@ -1618,19 +1637,19 @@
     </row>
     <row r="47" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>18</v>
@@ -1638,16 +1657,16 @@
     </row>
     <row r="48" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>6</v>
@@ -1658,22 +1677,22 @@
     </row>
     <row r="49" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1681,10 +1700,10 @@
         <v>2025</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>62</v>
+        <v>35</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>5</v>
@@ -1693,7 +1712,7 @@
         <v>6</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1701,10 +1720,10 @@
         <v>2025</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>11</v>
@@ -1718,16 +1737,16 @@
     </row>
     <row r="52" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>6</v>
@@ -1738,19 +1757,19 @@
     </row>
     <row r="53" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>18</v>
@@ -1758,13 +1777,13 @@
     </row>
     <row r="54" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>5</v>
@@ -1778,13 +1797,13 @@
     </row>
     <row r="55" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>11</v>
@@ -1801,13 +1820,13 @@
         <v>2026</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>6</v>
@@ -1821,13 +1840,13 @@
         <v>2026</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>12</v>
@@ -1841,18 +1860,158 @@
         <v>2026</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F58" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F65" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1862,6 +2021,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009DC89E0A0BD1B540A4E85B97489EFC3B" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="94867cae1703a82c97127efc4891e877">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2a2d371e-7a33-4a26-8ec1-44108789bebc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f3726ffbfb48ac77aba5882cc2e1bbd" ns2:_="">
     <xsd:import namespace="2a2d371e-7a33-4a26-8ec1-44108789bebc"/>
@@ -2033,15 +2201,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2053,15 +2212,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4A8F9B3-BD5E-4651-B37A-769458AD5BBA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2BB0C49-950B-4679-9E98-59899B5FC83D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2BB0C49-950B-4679-9E98-59899B5FC83D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4A8F9B3-BD5E-4651-B37A-769458AD5BBA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2a2d371e-7a33-4a26-8ec1-44108789bebc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30A0FF88-D728-43C4-8C63-4B9F337F27D5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30A0FF88-D728-43C4-8C63-4B9F337F27D5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2a2d371e-7a33-4a26-8ec1-44108789bebc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>